<commit_message>
Daily scans — 05-Jun-2026 23:19 — 19 file(s)
</commit_message>
<xml_diff>
--- a/Resilient_Stack_Reversal_2026-06-05.xlsx
+++ b/Resilient_Stack_Reversal_2026-06-05.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,12 +56,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="004A148C"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="13"/>
     </font>
@@ -94,7 +88,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -119,11 +113,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF9C4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EDE7F6"/>
       </patternFill>
     </fill>
     <fill>
@@ -198,21 +187,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -230,22 +219,19 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -636,7 +622,7 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>21-May-2026</t>
+          <t>05-Jun-2026</t>
         </is>
       </c>
     </row>
@@ -648,7 +634,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>07:02 IST</t>
+          <t>22:33 IST</t>
         </is>
       </c>
     </row>
@@ -980,52 +966,52 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>CARERATING</t>
+          <t>FIEMIND</t>
         </is>
       </c>
       <c r="C2" s="9" t="n">
         <v>84</v>
       </c>
       <c r="D2" s="7" t="n">
-        <v>1720.2</v>
+        <v>2311.2</v>
       </c>
       <c r="E2" s="7" t="n">
-        <v>3.6</v>
+        <v>3.3</v>
       </c>
       <c r="F2" s="7" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="G2" s="7" t="n">
-        <v>6</v>
+        <v>13.1</v>
+      </c>
+      <c r="G2" s="10" t="n">
+        <v>4</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>-3.93</v>
-      </c>
-      <c r="I2" s="10" t="n">
-        <v>4</v>
+        <v>-4.2</v>
+      </c>
+      <c r="I2" s="7" t="n">
+        <v>7</v>
       </c>
       <c r="J2" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="K2" s="11" t="n">
-        <v>0.33</v>
+      <c r="K2" s="10" t="n">
+        <v>2.19</v>
       </c>
       <c r="L2" s="7" t="n">
-        <v>8.33</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="M2" s="7" t="n">
-        <v>14.17</v>
+        <v>10.56</v>
       </c>
       <c r="N2" s="7" t="n">
-        <v>1651.39</v>
+        <v>2214.93</v>
       </c>
       <c r="O2" s="7" t="n">
-        <v>1622.17</v>
+        <v>2187.61</v>
       </c>
       <c r="P2" s="7" t="n">
-        <v>1587.93</v>
+        <v>2114.53</v>
       </c>
     </row>
   </sheetData>
@@ -1049,35 +1035,35 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="12" t="inlineStr">
-        <is>
-          <t>📺  TradingView Watchlist  —  21-May-2026  |  1 stocks</t>
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>📺  TradingView Watchlist  —  05-Jun-2026  |  1 stocks</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="13" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Click orange cell &gt;&gt; Ctrl+C &gt;&gt; TradingView &gt;&gt; Watchlist &gt;&gt; (...) &gt;&gt; Import List &gt;&gt; Paste</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  🛡 Resilient Reversal  —  1 stocks</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>1 symbols</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>NSE:CARERATING</t>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>NSE:FIEMIND</t>
         </is>
       </c>
     </row>

</xml_diff>